<commit_message>
Clean fake/template emails from results
Removed: mycompany@co.com, sample@domain.ru, privacy@thismywebsite.com,
coolwanglu@gmail.com (developer email, not clinic).
Final: 378/621 companies with real emails.

https://claude.ai/code/session_01RirjgdbnRw5p1vyEh4svFF
</commit_message>
<xml_diff>
--- a/companies_final.xlsx
+++ b/companies_final.xlsx
@@ -439,11 +439,7 @@
           <t>Детский центр нейропсихологии и канистерапии</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>mycompany@co.com</t>
-        </is>
-      </c>
+      <c r="E3" s="1" t="n"/>
     </row>
     <row r="4" ht="56" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
@@ -1570,11 +1566,7 @@
           <t>A Moscow-based child development center offering speech therapy, neurological interventions, and art/music therapy for children aged 2-18, with parental support and group sessions.</t>
         </is>
       </c>
-      <c r="E48" s="1" t="inlineStr">
-        <is>
-          <t>coolwanglu@gmail.com</t>
-        </is>
-      </c>
+      <c r="E48" s="1" t="n"/>
     </row>
     <row r="49" ht="56" customHeight="1">
       <c r="A49" s="1" t="inlineStr">
@@ -9220,11 +9212,7 @@
           <t>A Moscow-based children's learning center offering chess, math games, and creative activities for kids aged 2.5-14, with multiple locations and flexible scheduling.</t>
         </is>
       </c>
-      <c r="E350" s="1" t="inlineStr">
-        <is>
-          <t>sample@domain.ru</t>
-        </is>
-      </c>
+      <c r="E350" s="1" t="n"/>
     </row>
     <row r="351" ht="42" customHeight="1">
       <c r="A351" s="1" t="inlineStr">
@@ -10704,7 +10692,7 @@
       </c>
       <c r="E408" s="1" t="inlineStr">
         <is>
-          <t>lifemotion99@mail.ru, mycompany@co.com</t>
+          <t>lifemotion99@mail.ru</t>
         </is>
       </c>
     </row>
@@ -11868,11 +11856,7 @@
           <t>Clinical psychologist offering cognitive-behavioral therapy and existential analysis, specializing in trauma recovery and stress management through personalized counseling sessions.</t>
         </is>
       </c>
-      <c r="E454" s="1" t="inlineStr">
-        <is>
-          <t>privacy@thismywebsite.com</t>
-        </is>
-      </c>
+      <c r="E454" s="1" t="n"/>
     </row>
     <row r="455" ht="42" customHeight="1">
       <c r="A455" s="1" t="inlineStr">
@@ -16146,11 +16130,7 @@
           <t>Moscow preschool center preparing kids for school, located at Высотный проезд, with educational services via +7 (903) 709-99-66.</t>
         </is>
       </c>
-      <c r="E620" s="1" t="inlineStr">
-        <is>
-          <t>sample@domain.ru</t>
-        </is>
-      </c>
+      <c r="E620" s="1" t="n"/>
     </row>
     <row r="621" ht="56" customHeight="1">
       <c r="A621" s="1" t="inlineStr">

</xml_diff>